<commit_message>
Use full note weight per underlying in exposure analysis
Each underlying now carries the whole weight of every note it is in,
instead of the weight split equally across the basket.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XWZgcudBfQ6kiCtxuQQJeu
</commit_message>
<xml_diff>
--- a/analysis/underlying_exposure.xlsx
+++ b/analysis/underlying_exposure.xlsx
@@ -419,7 +419,7 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -508,11 +508,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Average new weight per underlying %</t>
+          <t>Average new exposure per underlying %</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.0075</v>
+        <v>2.8858</v>
       </c>
     </row>
     <row r="10">
@@ -528,11 +528,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Top 10 underlyings - new weight %</t>
+          <t>Top 10 underlyings - new exposure % (gross)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>23.63</v>
+        <v>67.09</v>
       </c>
     </row>
   </sheetData>
@@ -546,23 +546,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -588,7 +586,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Look-through EUR</t>
+          <t>Exposure EUR</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -622,16 +620,6 @@
         </is>
       </c>
       <c r="L1" t="inlineStr">
-        <is>
-          <t>Original gross %</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>New gross %</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t>Held via</t>
         </is>
@@ -657,35 +645,29 @@
         <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>633301.5943</v>
+        <v>1899904.783</v>
       </c>
       <c r="F2" t="n">
-        <v>3.6192</v>
+        <v>10.8575</v>
       </c>
       <c r="G2" t="n">
-        <v>3.378</v>
+        <v>10.1339</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.2412</v>
+        <v>-0.7235</v>
       </c>
       <c r="I2" t="n">
         <v>-6.664</v>
       </c>
       <c r="J2" t="n">
-        <v>2.3705</v>
+        <v>7.2481</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>10.8575</v>
-      </c>
-      <c r="M2" t="n">
-        <v>10.1339</v>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>HSBC AC 9% SPX-SX5E-NKY  01.12.2027; CITI AC 7.5% SPX-SX5E-SMI  07.02.2028; HSBC AC 7.75% SPX-NKY-SM  06.03.2028; UC AC 8.5% SPX-SX5E-NKY  04.11.2027</t>
         </is>
@@ -711,35 +693,29 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>509985.2339</v>
+        <v>1529955.7018</v>
       </c>
       <c r="F3" t="n">
-        <v>2.9144</v>
+        <v>8.7433</v>
       </c>
       <c r="G3" t="n">
-        <v>2.7202</v>
+        <v>8.160600000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1942</v>
+        <v>-0.5827</v>
       </c>
       <c r="I3" t="n">
         <v>-6.664</v>
       </c>
       <c r="J3" t="n">
-        <v>1.7127</v>
+        <v>5.2748</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>8.7433</v>
-      </c>
-      <c r="M3" t="n">
-        <v>8.160600000000001</v>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>POST AC 7.5% CAC-UKX-NDX  07.02.2028; BOFA AC 8.8% RTY-OMX-NDX  13.12.2027; CITI AC 8.5% NDX-RTY-SMI  25.01.2028</t>
         </is>
@@ -765,35 +741,29 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>500742.7546</v>
+        <v>1502228.2637</v>
       </c>
       <c r="F4" t="n">
-        <v>2.8616</v>
+        <v>8.5848</v>
       </c>
       <c r="G4" t="n">
-        <v>2.6709</v>
+        <v>8.012700000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1907</v>
+        <v>-0.5721000000000001</v>
       </c>
       <c r="I4" t="n">
         <v>-6.664</v>
       </c>
       <c r="J4" t="n">
-        <v>1.6634</v>
+        <v>5.1269</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>8.5848</v>
-      </c>
-      <c r="M4" t="n">
-        <v>8.012700000000001</v>
-      </c>
-      <c r="N4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>CITI AC 7.5% SPX-SX5E-SMI  07.02.2028; HSBC AC 7.75% SPX-NKY-SM  06.03.2028; CITI AC 8.5% NDX-RTY-SMI  25.01.2028</t>
         </is>
@@ -819,35 +789,29 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>488097.9496</v>
+        <v>1464293.8487</v>
       </c>
       <c r="F5" t="n">
-        <v>2.7894</v>
+        <v>8.3681</v>
       </c>
       <c r="G5" t="n">
-        <v>2.6035</v>
+        <v>7.8104</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1859</v>
+        <v>-0.5576</v>
       </c>
       <c r="I5" t="n">
         <v>-6.664</v>
       </c>
       <c r="J5" t="n">
-        <v>1.596</v>
+        <v>4.9246</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>8.3681</v>
-      </c>
-      <c r="M5" t="n">
-        <v>7.8104</v>
-      </c>
-      <c r="N5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>HSBC AC 9% SPX-SX5E-NKY  01.12.2027; HSBC AC 7.75% SPX-NKY-SM  06.03.2028; UC AC 8.5% SPX-SX5E-NKY  04.11.2027</t>
         </is>
@@ -873,35 +837,29 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>450349.5943</v>
+        <v>1351048.783</v>
       </c>
       <c r="F6" t="n">
-        <v>2.5736</v>
+        <v>7.7209</v>
       </c>
       <c r="G6" t="n">
-        <v>2.4021</v>
+        <v>7.2064</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1715</v>
+        <v>-0.5145</v>
       </c>
       <c r="I6" t="n">
         <v>-6.664</v>
       </c>
       <c r="J6" t="n">
-        <v>1.3946</v>
+        <v>4.3205</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>7.7209</v>
-      </c>
-      <c r="M6" t="n">
-        <v>7.2064</v>
-      </c>
-      <c r="N6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>HSBC AC 9% SPX-SX5E-NKY  01.12.2027; CITI AC 7.5% SPX-SX5E-SMI  07.02.2028; UC AC 8.5% SPX-SX5E-NKY  04.11.2027</t>
         </is>
@@ -910,12 +868,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Palo Alto Networks</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -924,40 +882,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>446979.9503</v>
+        <v>1066360.0811</v>
       </c>
       <c r="F7" t="n">
-        <v>2.5544</v>
+        <v>6.094</v>
       </c>
       <c r="G7" t="n">
-        <v>2.3841</v>
+        <v>5.6879</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1702</v>
+        <v>-0.4061</v>
       </c>
       <c r="I7" t="n">
         <v>-6.664</v>
       </c>
       <c r="J7" t="n">
-        <v>1.3767</v>
+        <v>2.802</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L7" t="n">
-        <v>4.2408</v>
-      </c>
-      <c r="M7" t="n">
-        <v>3.9582</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>GS AC 8.28% PANW  04.11.2027; UBS AC 9% PANW-SU-SIE  09.06.2027</t>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>TCM AC 9% AAPL-MSFT-AMZN  25.02.2027; JB AC 9% AAPL-GOOGL-AMZN  04.11.2027; STD AC 8% AMZN-MSFT-AAPL  18.04.2028</t>
         </is>
       </c>
     </row>
@@ -981,35 +933,29 @@
         <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>355453.3604</v>
+        <v>1066360.0811</v>
       </c>
       <c r="F8" t="n">
-        <v>2.0313</v>
+        <v>6.094</v>
       </c>
       <c r="G8" t="n">
-        <v>1.896</v>
+        <v>5.6879</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.1354</v>
+        <v>-0.4061</v>
       </c>
       <c r="I8" t="n">
         <v>-6.664</v>
       </c>
       <c r="J8" t="n">
-        <v>0.8885</v>
+        <v>2.802</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L8" t="n">
-        <v>6.094</v>
-      </c>
-      <c r="M8" t="n">
-        <v>5.6879</v>
-      </c>
-      <c r="N8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>TCM AC 9% AAPL-MSFT-AMZN  25.02.2027; JB AC 9% AAPL-GOOGL-AMZN  04.11.2027; STD AC 8% AMZN-MSFT-AAPL  18.04.2028</t>
         </is>
@@ -1018,120 +964,108 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Russell 2000</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Single stock</t>
+          <t>Index</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>355453.3604</v>
+        <v>1036805.7018</v>
       </c>
       <c r="F9" t="n">
-        <v>2.0313</v>
+        <v>5.9251</v>
       </c>
       <c r="G9" t="n">
-        <v>1.896</v>
+        <v>5.5302</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.1354</v>
+        <v>-0.3948</v>
       </c>
       <c r="I9" t="n">
         <v>-6.664</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8885</v>
+        <v>2.6444</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L9" t="n">
-        <v>6.094</v>
-      </c>
-      <c r="M9" t="n">
-        <v>5.6879</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>TCM AC 9% AAPL-MSFT-AMZN  25.02.2027; JB AC 9% AAPL-GOOGL-AMZN  04.11.2027; STD AC 8% AMZN-MSFT-AAPL  18.04.2028</t>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>BOFA AC 8.8% RTY-OMX-NDX  13.12.2027; CITI AC 8.5% NDX-RTY-SMI  25.01.2028</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Russell 2000</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Single stock</t>
         </is>
       </c>
       <c r="D10" t="n">
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>345601.9006</v>
+        <v>837836.8147</v>
       </c>
       <c r="F10" t="n">
-        <v>1.975</v>
+        <v>4.788</v>
       </c>
       <c r="G10" t="n">
-        <v>1.8434</v>
+        <v>4.4689</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.1316</v>
+        <v>-0.3191</v>
       </c>
       <c r="I10" t="n">
         <v>-6.664</v>
       </c>
       <c r="J10" t="n">
-        <v>0.8359</v>
+        <v>1.5831</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L10" t="n">
-        <v>5.9251</v>
-      </c>
-      <c r="M10" t="n">
-        <v>5.5302</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>BOFA AC 8.8% RTY-OMX-NDX  13.12.2027; CITI AC 8.5% NDX-RTY-SMI  25.01.2028</t>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>MS AC 8% TSM-META  05.01.2028; NAT AC 11% NVDA-TSM-ASML  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>Costco</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1143,49 +1077,43 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>344185.6049</v>
+        <v>822548</v>
       </c>
       <c r="F11" t="n">
-        <v>1.9669</v>
+        <v>4.7006</v>
       </c>
       <c r="G11" t="n">
-        <v>1.8359</v>
+        <v>4.3874</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.1311</v>
+        <v>-0.3133</v>
       </c>
       <c r="I11" t="n">
         <v>-6.664</v>
       </c>
       <c r="J11" t="n">
-        <v>0.8284</v>
+        <v>1.5016</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L11" t="n">
-        <v>4.788</v>
-      </c>
-      <c r="M11" t="n">
-        <v>4.4689</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>MS AC 8% TSM-META  05.01.2028; NAT AC 11% NVDA-TSM-ASML  04.11.2027</t>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>UBS AC 7% DE-COST-KO  07.02.2028; BOFA 8.5% AVGO-COST-GOOGL  08.03.2027</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Meta Platforms</t>
+          <t>Nvidia</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1197,49 +1125,43 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>327822.351</v>
+        <v>803372.0575999999</v>
       </c>
       <c r="F12" t="n">
-        <v>1.8734</v>
+        <v>4.5911</v>
       </c>
       <c r="G12" t="n">
-        <v>1.7486</v>
+        <v>4.2851</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.1248</v>
+        <v>-0.3059</v>
       </c>
       <c r="I12" t="n">
         <v>-6.664</v>
       </c>
       <c r="J12" t="n">
-        <v>0.7411</v>
+        <v>1.3993</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L12" t="n">
-        <v>3.7468</v>
-      </c>
-      <c r="M12" t="n">
-        <v>3.4971</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>STAN AC 10% AVGO-META  05.11.2027; MS AC 8% TSM-META  05.01.2028</t>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>OPUS AC 9% BKR-NVDA-ROG  04.03.2027; NAT AC 11% NVDA-TSM-ASML  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Broadcom</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1251,49 +1173,43 @@
         <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>275231.6844</v>
+        <v>776997.3325</v>
       </c>
       <c r="F13" t="n">
-        <v>1.5729</v>
+        <v>4.4403</v>
       </c>
       <c r="G13" t="n">
-        <v>1.4681</v>
+        <v>4.1444</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.1048</v>
+        <v>-0.2959</v>
       </c>
       <c r="I13" t="n">
         <v>-6.664</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4606</v>
+        <v>1.2586</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L13" t="n">
-        <v>3.958</v>
-      </c>
-      <c r="M13" t="n">
-        <v>3.6942</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>STAN AC 10% AVGO-META  05.11.2027; BOFA 8.5% AVGO-COST-GOOGL  08.03.2027</t>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>JB AC 9% AAPL-GOOGL-AMZN  04.11.2027; BOFA 8.5% AVGO-COST-GOOGL  08.03.2027</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>UBSG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Costco</t>
+          <t>UBS Group</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1305,49 +1221,43 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>274182.6667</v>
+        <v>751471.0368</v>
       </c>
       <c r="F14" t="n">
-        <v>1.5669</v>
+        <v>4.2945</v>
       </c>
       <c r="G14" t="n">
-        <v>1.4625</v>
+        <v>4.0083</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.1044</v>
+        <v>-0.2862</v>
       </c>
       <c r="I14" t="n">
         <v>-6.664</v>
       </c>
       <c r="J14" t="n">
-        <v>0.455</v>
+        <v>1.1225</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L14" t="n">
-        <v>4.7006</v>
-      </c>
-      <c r="M14" t="n">
-        <v>4.3874</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>UBS AC 7% DE-COST-KO  07.02.2028; BOFA 8.5% AVGO-COST-GOOGL  08.03.2027</t>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>POST AC 8.5% ABBN-NOVN-UB  29.09.2027; EFG AC 7% ZURN-V-UBSG  30.03.2028</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Palo Alto Networks</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1359,49 +1269,43 @@
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>267790.6859</v>
+        <v>742079.851</v>
       </c>
       <c r="F15" t="n">
-        <v>1.5304</v>
+        <v>4.2408</v>
       </c>
       <c r="G15" t="n">
-        <v>1.4284</v>
+        <v>3.9582</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.102</v>
+        <v>-0.2826</v>
       </c>
       <c r="I15" t="n">
         <v>-6.664</v>
       </c>
       <c r="J15" t="n">
-        <v>0.4209</v>
+        <v>1.0724</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L15" t="n">
-        <v>4.5911</v>
-      </c>
-      <c r="M15" t="n">
-        <v>4.2851</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>OPUS AC 9% BKR-NVDA-ROG  04.03.2027; NAT AC 11% NVDA-TSM-ASML  04.11.2027</t>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>GS AC 8.28% PANW  04.11.2027; UBS AC 9% PANW-SU-SIE  09.06.2027</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AIR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Airbus</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1413,49 +1317,43 @@
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>258999.1108</v>
+        <v>737285.7044</v>
       </c>
       <c r="F16" t="n">
-        <v>1.4801</v>
+        <v>4.2134</v>
       </c>
       <c r="G16" t="n">
-        <v>1.3815</v>
+        <v>3.9326</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.09859999999999999</v>
+        <v>-0.2808</v>
       </c>
       <c r="I16" t="n">
         <v>-6.664</v>
       </c>
       <c r="J16" t="n">
-        <v>0.374</v>
+        <v>1.0468</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L16" t="n">
-        <v>4.4403</v>
-      </c>
-      <c r="M16" t="n">
-        <v>4.1444</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>JB AC 9% AAPL-GOOGL-AMZN  04.11.2027; BOFA 8.5% AVGO-COST-GOOGL  08.03.2027</t>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>TCM AC 8.5% AIR-HNR1-LIN  18.11.2026; BIL AC 7.5% AIR-AM-SAF  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>UBSG</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>UBS Group</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1467,49 +1365,43 @@
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>250490.3456</v>
+        <v>717221.063</v>
       </c>
       <c r="F17" t="n">
-        <v>1.4315</v>
+        <v>4.0987</v>
       </c>
       <c r="G17" t="n">
-        <v>1.3361</v>
+        <v>3.8256</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.0954</v>
+        <v>-0.2731</v>
       </c>
       <c r="I17" t="n">
         <v>-6.664</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3286</v>
+        <v>0.9398</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L17" t="n">
-        <v>4.2945</v>
-      </c>
-      <c r="M17" t="n">
-        <v>4.0083</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>POST AC 8.5% ABBN-NOVN-UB  29.09.2027; EFG AC 7% ZURN-V-UBSG  30.03.2028</t>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>BIL AC 9.3% ASML-OR-DG  11.06.2027; NAT AC 11% NVDA-TSM-ASML  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1518,52 +1410,46 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>250000</v>
+        <v>716568.013</v>
       </c>
       <c r="F18" t="n">
-        <v>1.4287</v>
+        <v>4.095</v>
       </c>
       <c r="G18" t="n">
-        <v>1.3335</v>
+        <v>3.8221</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.09520000000000001</v>
+        <v>-0.2729</v>
       </c>
       <c r="I18" t="n">
         <v>-6.664</v>
       </c>
       <c r="J18" t="n">
-        <v>0.326</v>
+        <v>0.9363</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L18" t="n">
-        <v>2.8574</v>
-      </c>
-      <c r="M18" t="n">
-        <v>2.667</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>BOFA AC 8% AMD-TXN  31.12.2027</t>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>VO AC 8% HD-MA-WMT  01.03.2027; AKB AC 7.5% MCD-PG-WMT  22.03.2028</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1572,52 +1458,46 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>250000</v>
+        <v>715750.7486</v>
       </c>
       <c r="F19" t="n">
-        <v>1.4287</v>
+        <v>4.0903</v>
       </c>
       <c r="G19" t="n">
-        <v>1.3335</v>
+        <v>3.8177</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.09520000000000001</v>
+        <v>-0.2726</v>
       </c>
       <c r="I19" t="n">
         <v>-6.664</v>
       </c>
       <c r="J19" t="n">
-        <v>0.326</v>
+        <v>0.9319</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L19" t="n">
-        <v>2.8574</v>
-      </c>
-      <c r="M19" t="n">
-        <v>2.667</v>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>BOFA AC 8% AMD-TXN  31.12.2027</t>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>TCM AC 9% AAPL-MSFT-AMZN  25.02.2027; STD AC 8% AMZN-MSFT-AAPL  18.04.2028</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AIR</t>
+          <t>MCD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Airbus</t>
+          <t>McDonald's</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1629,49 +1509,43 @@
         <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>245761.9015</v>
+        <v>700529.975</v>
       </c>
       <c r="F20" t="n">
-        <v>1.4045</v>
+        <v>4.0033</v>
       </c>
       <c r="G20" t="n">
-        <v>1.3109</v>
+        <v>3.7366</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.0936</v>
+        <v>-0.2668</v>
       </c>
       <c r="I20" t="n">
         <v>-6.664</v>
       </c>
       <c r="J20" t="n">
-        <v>0.3034</v>
+        <v>0.8507</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L20" t="n">
-        <v>4.2134</v>
-      </c>
-      <c r="M20" t="n">
-        <v>3.9326</v>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>TCM AC 8.5% AIR-HNR1-LIN  18.11.2026; BIL AC 7.5% AIR-AM-SAF  04.11.2027</t>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>EFG AC 8.5% BKNG-CVX-MCD  01.03.2027; AKB AC 7.5% MCD-PG-WMT  22.03.2028</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>Broadcom</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1683,49 +1557,43 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>239073.6877</v>
+        <v>692592.7021</v>
       </c>
       <c r="F21" t="n">
-        <v>1.3662</v>
+        <v>3.958</v>
       </c>
       <c r="G21" t="n">
-        <v>1.2752</v>
+        <v>3.6942</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.091</v>
+        <v>-0.2638</v>
       </c>
       <c r="I21" t="n">
         <v>-6.664</v>
       </c>
       <c r="J21" t="n">
-        <v>0.2677</v>
+        <v>0.8084</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="L21" t="n">
-        <v>4.0987</v>
-      </c>
-      <c r="M21" t="n">
-        <v>3.8256</v>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>BIL AC 9.3% ASML-OR-DG  11.06.2027; NAT AC 11% NVDA-TSM-ASML  04.11.2027</t>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>STAN AC 10% AVGO-META  05.11.2027; BOFA 8.5% AVGO-COST-GOOGL  08.03.2027</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>L'Oreal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1737,49 +1605,43 @@
         <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>238856.0043</v>
+        <v>656784.2483</v>
       </c>
       <c r="F22" t="n">
-        <v>1.365</v>
+        <v>3.7534</v>
       </c>
       <c r="G22" t="n">
-        <v>1.274</v>
+        <v>3.5032</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.091</v>
+        <v>-0.2501</v>
       </c>
       <c r="I22" t="n">
         <v>-6.664</v>
       </c>
       <c r="J22" t="n">
-        <v>0.2666</v>
+        <v>0.6173999999999999</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Overweight</t>
-        </is>
-      </c>
-      <c r="L22" t="n">
-        <v>4.095</v>
-      </c>
-      <c r="M22" t="n">
-        <v>3.8221</v>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>VO AC 8% HD-MA-WMT  01.03.2027; AKB AC 7.5% MCD-PG-WMT  22.03.2028</t>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>BIL AC 9.3% ASML-OR-DG  11.06.2027; BIL AC 7% AI-OR-MC  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1791,49 +1653,43 @@
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>238583.5829</v>
+        <v>655644.7021</v>
       </c>
       <c r="F23" t="n">
-        <v>1.3634</v>
+        <v>3.7468</v>
       </c>
       <c r="G23" t="n">
-        <v>1.2726</v>
+        <v>3.4971</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.09089999999999999</v>
+        <v>-0.2497</v>
       </c>
       <c r="I23" t="n">
         <v>-6.664</v>
       </c>
       <c r="J23" t="n">
-        <v>0.2651</v>
+        <v>0.6113</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Overweight</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
-        <v>4.0903</v>
-      </c>
-      <c r="M23" t="n">
-        <v>3.8177</v>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>TCM AC 9% AAPL-MSFT-AMZN  25.02.2027; STD AC 8% AMZN-MSFT-AAPL  18.04.2028</t>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>STAN AC 10% AVGO-META  05.11.2027; MS AC 8% TSM-META  05.01.2028</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MCD</t>
+          <t>NOVN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>McDonald's</t>
+          <t>Novartis</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1845,49 +1701,43 @@
         <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>233509.9917</v>
+        <v>655209.3700999999</v>
       </c>
       <c r="F24" t="n">
-        <v>1.3344</v>
+        <v>3.7444</v>
       </c>
       <c r="G24" t="n">
-        <v>1.2455</v>
+        <v>3.4948</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.08890000000000001</v>
+        <v>-0.2495</v>
       </c>
       <c r="I24" t="n">
         <v>-6.664</v>
       </c>
       <c r="J24" t="n">
-        <v>0.238</v>
+        <v>0.609</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L24" t="n">
-        <v>4.0033</v>
-      </c>
-      <c r="M24" t="n">
-        <v>3.7366</v>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>EFG AC 8.5% BKNG-CVX-MCD  01.03.2027; AKB AC 7.5% MCD-PG-WMT  22.03.2028</t>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>POST AC 8.5% ABBN-NOVN-UB  29.09.2027; BNP AC 7% LLY-MRK-NOVN  05.01.2028</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>L'Oreal</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1899,103 +1749,91 @@
         <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>218928.0828</v>
+        <v>565697.2432</v>
       </c>
       <c r="F25" t="n">
-        <v>1.2511</v>
+        <v>3.2328</v>
       </c>
       <c r="G25" t="n">
-        <v>1.1677</v>
+        <v>3.0174</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.0834</v>
+        <v>-0.2154</v>
       </c>
       <c r="I25" t="n">
         <v>-6.664</v>
       </c>
       <c r="J25" t="n">
-        <v>0.1603</v>
+        <v>0.1316</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L25" t="n">
-        <v>3.7534</v>
-      </c>
-      <c r="M25" t="n">
-        <v>3.5032</v>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>BIL AC 9.3% ASML-OR-DG  11.06.2027; BIL AC 7% AI-OR-MC  04.11.2027</t>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>VO AC 8% HD-MA-WMT  01.03.2027; VO AC 8.5% UBER-JPM-MA  01.02.2027</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NOVN</t>
+          <t>OMX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Novartis</t>
+          <t>OMX Stockholm 30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Single stock</t>
+          <t>Index</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>218403.1234</v>
+        <v>519044.3724</v>
       </c>
       <c r="F26" t="n">
-        <v>1.2481</v>
+        <v>2.9662</v>
       </c>
       <c r="G26" t="n">
-        <v>1.1649</v>
+        <v>2.7685</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.0832</v>
+        <v>-0.1977</v>
       </c>
       <c r="I26" t="n">
         <v>-6.664</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1575</v>
+        <v>-0.1173</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L26" t="n">
-        <v>3.7444</v>
-      </c>
-      <c r="M26" t="n">
-        <v>3.4948</v>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>POST AC 8.5% ABBN-NOVN-UB  29.09.2027; BNP AC 7% LLY-MRK-NOVN  05.01.2028</t>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>BOFA AC 8.8% RTY-OMX-NDX  13.12.2027</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2004,106 +1842,94 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>188565.7477</v>
+        <v>500500</v>
       </c>
       <c r="F27" t="n">
-        <v>1.0776</v>
+        <v>2.8602</v>
       </c>
       <c r="G27" t="n">
-        <v>1.0058</v>
+        <v>2.6696</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.0718</v>
+        <v>-0.1906</v>
       </c>
       <c r="I27" t="n">
         <v>-6.664</v>
       </c>
       <c r="J27" t="n">
-        <v>-0.0017</v>
+        <v>-0.2162</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L27" t="n">
-        <v>3.2328</v>
-      </c>
-      <c r="M27" t="n">
-        <v>3.0174</v>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>VO AC 8% HD-MA-WMT  01.03.2027; VO AC 8.5% UBER-JPM-MA  01.02.2027</t>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>AKB AC 7.5% MCD-PG-WMT  22.03.2028</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OMX</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OMX Stockholm 30</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Single stock</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>173014.7908</v>
+        <v>500000</v>
       </c>
       <c r="F28" t="n">
-        <v>0.9887</v>
+        <v>2.8574</v>
       </c>
       <c r="G28" t="n">
-        <v>0.9228</v>
+        <v>2.667</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.0659</v>
+        <v>-0.1904</v>
       </c>
       <c r="I28" t="n">
         <v>-6.664</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.08459999999999999</v>
+        <v>-0.2189</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L28" t="n">
-        <v>2.9662</v>
-      </c>
-      <c r="M28" t="n">
-        <v>2.7685</v>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>BOFA AC 8.8% RTY-OMX-NDX  13.12.2027</t>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>BOFA AC 8% AMD-TXN  31.12.2027</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2115,37 +1941,31 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>166833.3333</v>
+        <v>500000</v>
       </c>
       <c r="F29" t="n">
-        <v>0.9534</v>
+        <v>2.8574</v>
       </c>
       <c r="G29" t="n">
-        <v>0.8899</v>
+        <v>2.667</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.0635</v>
+        <v>-0.1904</v>
       </c>
       <c r="I29" t="n">
         <v>-6.664</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.1176</v>
+        <v>-0.2189</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L29" t="n">
-        <v>2.8602</v>
-      </c>
-      <c r="M29" t="n">
-        <v>2.6696</v>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>AKB AC 7.5% MCD-PG-WMT  22.03.2028</t>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>BOFA AC 8% AMD-TXN  31.12.2027</t>
         </is>
       </c>
     </row>
@@ -2169,35 +1989,29 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>164847.2222</v>
+        <v>494541.6667</v>
       </c>
       <c r="F30" t="n">
-        <v>0.9421</v>
+        <v>2.8262</v>
       </c>
       <c r="G30" t="n">
-        <v>0.8793</v>
+        <v>2.6378</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.06279999999999999</v>
+        <v>-0.1883</v>
       </c>
       <c r="I30" t="n">
         <v>-6.664</v>
       </c>
       <c r="J30" t="n">
-        <v>-0.1282</v>
+        <v>-0.248</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L30" t="n">
-        <v>2.8262</v>
-      </c>
-      <c r="M30" t="n">
-        <v>2.6378</v>
-      </c>
-      <c r="N30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>EFG AC 7% ZURN-V-UBSG  30.03.2028</t>
         </is>
@@ -2223,35 +2037,29 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>164847.2222</v>
+        <v>494541.6667</v>
       </c>
       <c r="F31" t="n">
-        <v>0.9421</v>
+        <v>2.8262</v>
       </c>
       <c r="G31" t="n">
-        <v>0.8793</v>
+        <v>2.6378</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.06279999999999999</v>
+        <v>-0.1883</v>
       </c>
       <c r="I31" t="n">
         <v>-6.664</v>
       </c>
       <c r="J31" t="n">
-        <v>-0.1282</v>
+        <v>-0.248</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L31" t="n">
-        <v>2.8262</v>
-      </c>
-      <c r="M31" t="n">
-        <v>2.6378</v>
-      </c>
-      <c r="N31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>EFG AC 7% ZURN-V-UBSG  30.03.2028</t>
         </is>
@@ -2277,35 +2085,29 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>164750</v>
+        <v>494250</v>
       </c>
       <c r="F32" t="n">
-        <v>0.9415</v>
+        <v>2.8245</v>
       </c>
       <c r="G32" t="n">
-        <v>0.8788</v>
+        <v>2.6363</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.06270000000000001</v>
+        <v>-0.1882</v>
       </c>
       <c r="I32" t="n">
         <v>-6.664</v>
       </c>
       <c r="J32" t="n">
-        <v>-0.1287</v>
+        <v>-0.2495</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L32" t="n">
-        <v>2.8245</v>
-      </c>
-      <c r="M32" t="n">
-        <v>2.6363</v>
-      </c>
-      <c r="N32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>GS AC 8% ENR-RWE-TTE  04.08.2027</t>
         </is>
@@ -2331,35 +2133,29 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>164750</v>
+        <v>494250</v>
       </c>
       <c r="F33" t="n">
-        <v>0.9415</v>
+        <v>2.8245</v>
       </c>
       <c r="G33" t="n">
-        <v>0.8788</v>
+        <v>2.6363</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.06270000000000001</v>
+        <v>-0.1882</v>
       </c>
       <c r="I33" t="n">
         <v>-6.664</v>
       </c>
       <c r="J33" t="n">
-        <v>-0.1287</v>
+        <v>-0.2495</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L33" t="n">
-        <v>2.8245</v>
-      </c>
-      <c r="M33" t="n">
-        <v>2.6363</v>
-      </c>
-      <c r="N33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>GS AC 8% ENR-RWE-TTE  04.08.2027</t>
         </is>
@@ -2385,35 +2181,29 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>164750</v>
+        <v>494250</v>
       </c>
       <c r="F34" t="n">
-        <v>0.9415</v>
+        <v>2.8245</v>
       </c>
       <c r="G34" t="n">
-        <v>0.8788</v>
+        <v>2.6363</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.06270000000000001</v>
+        <v>-0.1882</v>
       </c>
       <c r="I34" t="n">
         <v>-6.664</v>
       </c>
       <c r="J34" t="n">
-        <v>-0.1287</v>
+        <v>-0.2495</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L34" t="n">
-        <v>2.8245</v>
-      </c>
-      <c r="M34" t="n">
-        <v>2.6363</v>
-      </c>
-      <c r="N34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>GS AC 8% ENR-RWE-TTE  04.08.2027</t>
         </is>
@@ -2439,35 +2229,29 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>164383.3333</v>
+        <v>493150</v>
       </c>
       <c r="F35" t="n">
-        <v>0.9394</v>
+        <v>2.8182</v>
       </c>
       <c r="G35" t="n">
-        <v>0.8768</v>
+        <v>2.6304</v>
       </c>
       <c r="H35" t="n">
-        <v>-0.0626</v>
+        <v>-0.1878</v>
       </c>
       <c r="I35" t="n">
         <v>-6.664</v>
       </c>
       <c r="J35" t="n">
-        <v>-0.1307</v>
+        <v>-0.2554</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L35" t="n">
-        <v>2.8182</v>
-      </c>
-      <c r="M35" t="n">
-        <v>2.6304</v>
-      </c>
-      <c r="N35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>POST AC 7.5% CAC-UKX-NDX  07.02.2028</t>
         </is>
@@ -2493,35 +2277,29 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>164383.3333</v>
+        <v>493150</v>
       </c>
       <c r="F36" t="n">
-        <v>0.9394</v>
+        <v>2.8182</v>
       </c>
       <c r="G36" t="n">
-        <v>0.8768</v>
+        <v>2.6304</v>
       </c>
       <c r="H36" t="n">
-        <v>-0.0626</v>
+        <v>-0.1878</v>
       </c>
       <c r="I36" t="n">
         <v>-6.664</v>
       </c>
       <c r="J36" t="n">
-        <v>-0.1307</v>
+        <v>-0.2554</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L36" t="n">
-        <v>2.8182</v>
-      </c>
-      <c r="M36" t="n">
-        <v>2.6304</v>
-      </c>
-      <c r="N36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>POST AC 7.5% CAC-UKX-NDX  07.02.2028</t>
         </is>
@@ -2547,35 +2325,29 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>158057.8353</v>
+        <v>474173.5059</v>
       </c>
       <c r="F37" t="n">
-        <v>0.9033</v>
+        <v>2.7098</v>
       </c>
       <c r="G37" t="n">
-        <v>0.8431</v>
+        <v>2.5292</v>
       </c>
       <c r="H37" t="n">
-        <v>-0.0602</v>
+        <v>-0.1806</v>
       </c>
       <c r="I37" t="n">
         <v>-6.664</v>
       </c>
       <c r="J37" t="n">
-        <v>-0.1644</v>
+        <v>-0.3566</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L37" t="n">
-        <v>2.7098</v>
-      </c>
-      <c r="M37" t="n">
-        <v>2.5292</v>
-      </c>
-      <c r="N37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>RAF AC 9% BNP-GS-MS  04.11.2027</t>
         </is>
@@ -2601,35 +2373,29 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>158057.8353</v>
+        <v>474173.5059</v>
       </c>
       <c r="F38" t="n">
-        <v>0.9033</v>
+        <v>2.7098</v>
       </c>
       <c r="G38" t="n">
-        <v>0.8431</v>
+        <v>2.5292</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.0602</v>
+        <v>-0.1806</v>
       </c>
       <c r="I38" t="n">
         <v>-6.664</v>
       </c>
       <c r="J38" t="n">
-        <v>-0.1644</v>
+        <v>-0.3566</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L38" t="n">
-        <v>2.7098</v>
-      </c>
-      <c r="M38" t="n">
-        <v>2.5292</v>
-      </c>
-      <c r="N38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>RAF AC 9% BNP-GS-MS  04.11.2027</t>
         </is>
@@ -2655,35 +2421,29 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>158057.8353</v>
+        <v>474173.5059</v>
       </c>
       <c r="F39" t="n">
-        <v>0.9033</v>
+        <v>2.7098</v>
       </c>
       <c r="G39" t="n">
-        <v>0.8431</v>
+        <v>2.5292</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.0602</v>
+        <v>-0.1806</v>
       </c>
       <c r="I39" t="n">
         <v>-6.664</v>
       </c>
       <c r="J39" t="n">
-        <v>-0.1644</v>
+        <v>-0.3566</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L39" t="n">
-        <v>2.7098</v>
-      </c>
-      <c r="M39" t="n">
-        <v>2.5292</v>
-      </c>
-      <c r="N39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>RAF AC 9% BNP-GS-MS  04.11.2027</t>
         </is>
@@ -2709,35 +2469,29 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>147549.9503</v>
+        <v>442649.851</v>
       </c>
       <c r="F40" t="n">
-        <v>0.8431999999999999</v>
+        <v>2.5296</v>
       </c>
       <c r="G40" t="n">
-        <v>0.787</v>
+        <v>2.3611</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.0562</v>
+        <v>-0.1686</v>
       </c>
       <c r="I40" t="n">
         <v>-6.664</v>
       </c>
       <c r="J40" t="n">
-        <v>-0.2205</v>
+        <v>-0.5248</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L40" t="n">
-        <v>2.5296</v>
-      </c>
-      <c r="M40" t="n">
-        <v>2.3611</v>
-      </c>
-      <c r="N40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>UBS AC 9% PANW-SU-SIE  09.06.2027</t>
         </is>
@@ -2763,35 +2517,29 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>147549.9503</v>
+        <v>442649.851</v>
       </c>
       <c r="F41" t="n">
-        <v>0.8431999999999999</v>
+        <v>2.5296</v>
       </c>
       <c r="G41" t="n">
-        <v>0.787</v>
+        <v>2.3611</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.0562</v>
+        <v>-0.1686</v>
       </c>
       <c r="I41" t="n">
         <v>-6.664</v>
       </c>
       <c r="J41" t="n">
-        <v>-0.2205</v>
+        <v>-0.5248</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="L41" t="n">
-        <v>2.5296</v>
-      </c>
-      <c r="M41" t="n">
-        <v>2.3611</v>
-      </c>
-      <c r="N41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>UBS AC 9% PANW-SU-SIE  09.06.2027</t>
         </is>
@@ -2800,120 +2548,108 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Arista Networks</t>
+          <t>Global X Uranium</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Single stock</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="D42" t="n">
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>134438.8542</v>
+        <v>399026.3875</v>
       </c>
       <c r="F42" t="n">
-        <v>0.7683</v>
+        <v>2.2803</v>
       </c>
       <c r="G42" t="n">
-        <v>0.7171</v>
+        <v>2.1284</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.0512</v>
+        <v>-0.152</v>
       </c>
       <c r="I42" t="n">
         <v>-6.664</v>
       </c>
       <c r="J42" t="n">
-        <v>-0.2904</v>
+        <v>-0.7575</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L42" t="n">
-        <v>1.5366</v>
-      </c>
-      <c r="M42" t="n">
-        <v>1.4342</v>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>UBS AC 11.1% ANET-APH  04.08.2027</t>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>NAT AC 9% GDX-COPX-URA  04.08.2027</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Amphenol</t>
+          <t>VanEck Gold Miners</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Single stock</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>134438.8542</v>
+        <v>399026.3875</v>
       </c>
       <c r="F43" t="n">
-        <v>0.7683</v>
+        <v>2.2803</v>
       </c>
       <c r="G43" t="n">
-        <v>0.7171</v>
+        <v>2.1284</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.0512</v>
+        <v>-0.152</v>
       </c>
       <c r="I43" t="n">
         <v>-6.664</v>
       </c>
       <c r="J43" t="n">
-        <v>-0.2904</v>
+        <v>-0.7575</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L43" t="n">
-        <v>1.5366</v>
-      </c>
-      <c r="M43" t="n">
-        <v>1.4342</v>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>UBS AC 11.1% ANET-APH  04.08.2027</t>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>NAT AC 9% GDX-COPX-URA  04.08.2027</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>COPX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>VanEck Gold Miners</t>
+          <t>Global X Copper Miners</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2925,35 +2661,29 @@
         <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>133008.7958</v>
+        <v>399026.3875</v>
       </c>
       <c r="F44" t="n">
-        <v>0.7601</v>
+        <v>2.2803</v>
       </c>
       <c r="G44" t="n">
-        <v>0.7095</v>
+        <v>2.1284</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.0507</v>
+        <v>-0.152</v>
       </c>
       <c r="I44" t="n">
         <v>-6.664</v>
       </c>
       <c r="J44" t="n">
-        <v>-0.298</v>
+        <v>-0.7575</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L44" t="n">
-        <v>2.2803</v>
-      </c>
-      <c r="M44" t="n">
-        <v>2.1284</v>
-      </c>
-      <c r="N44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>NAT AC 9% GDX-COPX-URA  04.08.2027</t>
         </is>
@@ -2962,120 +2692,108 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Global X Uranium</t>
+          <t>Merck &amp; Co</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ETF</t>
+          <t>Single stock</t>
         </is>
       </c>
       <c r="D45" t="n">
         <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>133008.7958</v>
+        <v>398280</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7601</v>
+        <v>2.2761</v>
       </c>
       <c r="G45" t="n">
-        <v>0.7095</v>
+        <v>2.1244</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.0507</v>
+        <v>-0.1517</v>
       </c>
       <c r="I45" t="n">
         <v>-6.664</v>
       </c>
       <c r="J45" t="n">
-        <v>-0.298</v>
+        <v>-0.7614</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L45" t="n">
-        <v>2.2803</v>
-      </c>
-      <c r="M45" t="n">
-        <v>2.1284</v>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>NAT AC 9% GDX-COPX-URA  04.08.2027</t>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>BNP AC 7% LLY-MRK-NOVN  05.01.2028</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>COPX</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Global X Copper Miners</t>
+          <t>Eli Lilly</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ETF</t>
+          <t>Single stock</t>
         </is>
       </c>
       <c r="D46" t="n">
         <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>133008.7958</v>
+        <v>398280</v>
       </c>
       <c r="F46" t="n">
-        <v>0.7601</v>
+        <v>2.2761</v>
       </c>
       <c r="G46" t="n">
-        <v>0.7095</v>
+        <v>2.1244</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.0507</v>
+        <v>-0.1517</v>
       </c>
       <c r="I46" t="n">
         <v>-6.664</v>
       </c>
       <c r="J46" t="n">
-        <v>-0.298</v>
+        <v>-0.7614</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L46" t="n">
-        <v>2.2803</v>
-      </c>
-      <c r="M46" t="n">
-        <v>2.1284</v>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>NAT AC 9% GDX-COPX-URA  04.08.2027</t>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>BNP AC 7% LLY-MRK-NOVN  05.01.2028</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Merck &amp; Co</t>
+          <t>Coca-Cola</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3087,49 +2805,43 @@
         <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>132760</v>
+        <v>396160</v>
       </c>
       <c r="F47" t="n">
-        <v>0.7587</v>
+        <v>2.264</v>
       </c>
       <c r="G47" t="n">
-        <v>0.7081</v>
+        <v>2.1131</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.0506</v>
+        <v>-0.1509</v>
       </c>
       <c r="I47" t="n">
         <v>-6.664</v>
       </c>
       <c r="J47" t="n">
-        <v>-0.2994</v>
+        <v>-0.7727000000000001</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L47" t="n">
-        <v>2.2761</v>
-      </c>
-      <c r="M47" t="n">
-        <v>2.1244</v>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>BNP AC 7% LLY-MRK-NOVN  05.01.2028</t>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>UBS AC 7% DE-COST-KO  07.02.2028</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Eli Lilly</t>
+          <t>Deere</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3141,49 +2853,43 @@
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>132760</v>
+        <v>396160</v>
       </c>
       <c r="F48" t="n">
-        <v>0.7587</v>
+        <v>2.264</v>
       </c>
       <c r="G48" t="n">
-        <v>0.7081</v>
+        <v>2.1131</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.0506</v>
+        <v>-0.1509</v>
       </c>
       <c r="I48" t="n">
         <v>-6.664</v>
       </c>
       <c r="J48" t="n">
-        <v>-0.2994</v>
+        <v>-0.7727000000000001</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L48" t="n">
-        <v>2.2761</v>
-      </c>
-      <c r="M48" t="n">
-        <v>2.1244</v>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>BNP AC 7% LLY-MRK-NOVN  05.01.2028</t>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>UBS AC 7% DE-COST-KO  07.02.2028</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>HO</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Coca-Cola</t>
+          <t>Thales</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3195,49 +2901,43 @@
         <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>132053.3333</v>
+        <v>392000</v>
       </c>
       <c r="F49" t="n">
-        <v>0.7547</v>
+        <v>2.2402</v>
       </c>
       <c r="G49" t="n">
-        <v>0.7044</v>
+        <v>2.0909</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.0503</v>
+        <v>-0.1493</v>
       </c>
       <c r="I49" t="n">
         <v>-6.664</v>
       </c>
       <c r="J49" t="n">
-        <v>-0.3031</v>
+        <v>-0.7949000000000001</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L49" t="n">
-        <v>2.264</v>
-      </c>
-      <c r="M49" t="n">
-        <v>2.1131</v>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>UBS AC 7% DE-COST-KO  07.02.2028</t>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>GS AC 7% RHM-RTX-HO  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Deere</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3249,49 +2949,43 @@
         <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>132053.3333</v>
+        <v>392000</v>
       </c>
       <c r="F50" t="n">
-        <v>0.7547</v>
+        <v>2.2402</v>
       </c>
       <c r="G50" t="n">
-        <v>0.7044</v>
+        <v>2.0909</v>
       </c>
       <c r="H50" t="n">
-        <v>-0.0503</v>
+        <v>-0.1493</v>
       </c>
       <c r="I50" t="n">
         <v>-6.664</v>
       </c>
       <c r="J50" t="n">
-        <v>-0.3031</v>
+        <v>-0.7949000000000001</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L50" t="n">
-        <v>2.264</v>
-      </c>
-      <c r="M50" t="n">
-        <v>2.1131</v>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>UBS AC 7% DE-COST-KO  07.02.2028</t>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>GS AC 7% RHM-RTX-HO  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>RHM</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Thales</t>
+          <t>Rheinmetall</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3303,35 +2997,29 @@
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>130666.6667</v>
+        <v>392000</v>
       </c>
       <c r="F51" t="n">
-        <v>0.7467</v>
+        <v>2.2402</v>
       </c>
       <c r="G51" t="n">
-        <v>0.697</v>
+        <v>2.0909</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.0498</v>
+        <v>-0.1493</v>
       </c>
       <c r="I51" t="n">
         <v>-6.664</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.3105</v>
+        <v>-0.7949000000000001</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L51" t="n">
-        <v>2.2402</v>
-      </c>
-      <c r="M51" t="n">
-        <v>2.0909</v>
-      </c>
-      <c r="N51" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>GS AC 7% RHM-RTX-HO  04.11.2027</t>
         </is>
@@ -3340,12 +3028,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3357,49 +3045,43 @@
         <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>130666.6667</v>
+        <v>391240</v>
       </c>
       <c r="F52" t="n">
-        <v>0.7467</v>
+        <v>2.2358</v>
       </c>
       <c r="G52" t="n">
-        <v>0.697</v>
+        <v>2.0868</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.0498</v>
+        <v>-0.149</v>
       </c>
       <c r="I52" t="n">
         <v>-6.664</v>
       </c>
       <c r="J52" t="n">
-        <v>-0.3105</v>
+        <v>-0.799</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L52" t="n">
-        <v>2.2402</v>
-      </c>
-      <c r="M52" t="n">
-        <v>2.0909</v>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>GS AC 7% RHM-RTX-HO  04.11.2027</t>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>CITI AC 7% AZN-JNJ-MCK  07.02.2028</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RHM</t>
+          <t>MCK</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Rheinmetall</t>
+          <t>McKesson</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3411,49 +3093,43 @@
         <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>130666.6667</v>
+        <v>391240</v>
       </c>
       <c r="F53" t="n">
-        <v>0.7467</v>
+        <v>2.2358</v>
       </c>
       <c r="G53" t="n">
-        <v>0.697</v>
+        <v>2.0868</v>
       </c>
       <c r="H53" t="n">
-        <v>-0.0498</v>
+        <v>-0.149</v>
       </c>
       <c r="I53" t="n">
         <v>-6.664</v>
       </c>
       <c r="J53" t="n">
-        <v>-0.3105</v>
+        <v>-0.799</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L53" t="n">
-        <v>2.2402</v>
-      </c>
-      <c r="M53" t="n">
-        <v>2.0909</v>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>GS AC 7% RHM-RTX-HO  04.11.2027</t>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>CITI AC 7% AZN-JNJ-MCK  07.02.2028</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MCK</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>McKesson</t>
+          <t>Johnson &amp; Johnson</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3465,35 +3141,29 @@
         <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>130413.3333</v>
+        <v>391240</v>
       </c>
       <c r="F54" t="n">
-        <v>0.7453</v>
+        <v>2.2358</v>
       </c>
       <c r="G54" t="n">
-        <v>0.6956</v>
+        <v>2.0868</v>
       </c>
       <c r="H54" t="n">
-        <v>-0.0497</v>
+        <v>-0.149</v>
       </c>
       <c r="I54" t="n">
         <v>-6.664</v>
       </c>
       <c r="J54" t="n">
-        <v>-0.3119</v>
+        <v>-0.799</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L54" t="n">
-        <v>2.2358</v>
-      </c>
-      <c r="M54" t="n">
-        <v>2.0868</v>
-      </c>
-      <c r="N54" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>CITI AC 7% AZN-JNJ-MCK  07.02.2028</t>
         </is>
@@ -3502,12 +3172,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>SAF</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>Safran</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3519,49 +3189,43 @@
         <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>130413.3333</v>
+        <v>390080</v>
       </c>
       <c r="F55" t="n">
-        <v>0.7453</v>
+        <v>2.2292</v>
       </c>
       <c r="G55" t="n">
-        <v>0.6956</v>
+        <v>2.0807</v>
       </c>
       <c r="H55" t="n">
-        <v>-0.0497</v>
+        <v>-0.1486</v>
       </c>
       <c r="I55" t="n">
         <v>-6.664</v>
       </c>
       <c r="J55" t="n">
-        <v>-0.3119</v>
+        <v>-0.8052</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L55" t="n">
-        <v>2.2358</v>
-      </c>
-      <c r="M55" t="n">
-        <v>2.0868</v>
-      </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>CITI AC 7% AZN-JNJ-MCK  07.02.2028</t>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>BIL AC 7.5% AIR-AM-SAF  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Johnson &amp; Johnson</t>
+          <t>Dassault Aviation</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3573,49 +3237,43 @@
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>130413.3333</v>
+        <v>390080</v>
       </c>
       <c r="F56" t="n">
-        <v>0.7453</v>
+        <v>2.2292</v>
       </c>
       <c r="G56" t="n">
-        <v>0.6956</v>
+        <v>2.0807</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.0497</v>
+        <v>-0.1486</v>
       </c>
       <c r="I56" t="n">
         <v>-6.664</v>
       </c>
       <c r="J56" t="n">
-        <v>-0.3119</v>
+        <v>-0.8052</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L56" t="n">
-        <v>2.2358</v>
-      </c>
-      <c r="M56" t="n">
-        <v>2.0868</v>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>CITI AC 7% AZN-JNJ-MCK  07.02.2028</t>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>BIL AC 7.5% AIR-AM-SAF  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SAF</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Safran</t>
+          <t>Air Liquide</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3627,49 +3285,43 @@
         <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>130026.6667</v>
+        <v>387960</v>
       </c>
       <c r="F57" t="n">
-        <v>0.7431</v>
+        <v>2.2171</v>
       </c>
       <c r="G57" t="n">
-        <v>0.6936</v>
+        <v>2.0693</v>
       </c>
       <c r="H57" t="n">
-        <v>-0.0495</v>
+        <v>-0.1477</v>
       </c>
       <c r="I57" t="n">
         <v>-6.664</v>
       </c>
       <c r="J57" t="n">
-        <v>-0.3139</v>
+        <v>-0.8165</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L57" t="n">
-        <v>2.2292</v>
-      </c>
-      <c r="M57" t="n">
-        <v>2.0807</v>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>BIL AC 7.5% AIR-AM-SAF  04.11.2027</t>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>BIL AC 7% AI-OR-MC  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dassault Aviation</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3681,49 +3333,43 @@
         <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>130026.6667</v>
+        <v>387960</v>
       </c>
       <c r="F58" t="n">
-        <v>0.7431</v>
+        <v>2.2171</v>
       </c>
       <c r="G58" t="n">
-        <v>0.6936</v>
+        <v>2.0693</v>
       </c>
       <c r="H58" t="n">
-        <v>-0.0495</v>
+        <v>-0.1477</v>
       </c>
       <c r="I58" t="n">
         <v>-6.664</v>
       </c>
       <c r="J58" t="n">
-        <v>-0.3139</v>
+        <v>-0.8165</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L58" t="n">
-        <v>2.2292</v>
-      </c>
-      <c r="M58" t="n">
-        <v>2.0807</v>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>BIL AC 7.5% AIR-AM-SAF  04.11.2027</t>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>BIL AC 7% AI-OR-MC  04.11.2027</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Air Liquide</t>
+          <t>Baker Hughes</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3735,49 +3381,43 @@
         <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>129320</v>
+        <v>354975.2429</v>
       </c>
       <c r="F59" t="n">
-        <v>0.739</v>
+        <v>2.0286</v>
       </c>
       <c r="G59" t="n">
-        <v>0.6898</v>
+        <v>1.8934</v>
       </c>
       <c r="H59" t="n">
-        <v>-0.0492</v>
+        <v>-0.1352</v>
       </c>
       <c r="I59" t="n">
         <v>-6.664</v>
       </c>
       <c r="J59" t="n">
-        <v>-0.3177</v>
+        <v>-0.9923999999999999</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L59" t="n">
-        <v>2.2171</v>
-      </c>
-      <c r="M59" t="n">
-        <v>2.0693</v>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>BIL AC 7% AI-OR-MC  04.11.2027</t>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>OPUS AC 9% BKR-NVDA-ROG  04.03.2027</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>ROG</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3789,49 +3429,43 @@
         <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>129320</v>
+        <v>354975.2429</v>
       </c>
       <c r="F60" t="n">
-        <v>0.739</v>
+        <v>2.0286</v>
       </c>
       <c r="G60" t="n">
-        <v>0.6898</v>
+        <v>1.8934</v>
       </c>
       <c r="H60" t="n">
-        <v>-0.0492</v>
+        <v>-0.1352</v>
       </c>
       <c r="I60" t="n">
         <v>-6.664</v>
       </c>
       <c r="J60" t="n">
-        <v>-0.3177</v>
+        <v>-0.9923999999999999</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L60" t="n">
-        <v>2.2171</v>
-      </c>
-      <c r="M60" t="n">
-        <v>2.0693</v>
-      </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>BIL AC 7% AI-OR-MC  04.11.2027</t>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>OPUS AC 9% BKR-NVDA-ROG  04.03.2027</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BKR</t>
+          <t>UBER</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Baker Hughes</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3843,49 +3477,43 @@
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>118325.081</v>
+        <v>349629.2302</v>
       </c>
       <c r="F61" t="n">
-        <v>0.6762</v>
+        <v>1.998</v>
       </c>
       <c r="G61" t="n">
-        <v>0.6311</v>
+        <v>1.8649</v>
       </c>
       <c r="H61" t="n">
-        <v>-0.0451</v>
+        <v>-0.1331</v>
       </c>
       <c r="I61" t="n">
         <v>-6.664</v>
       </c>
       <c r="J61" t="n">
-        <v>-0.3763</v>
+        <v>-1.0209</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L61" t="n">
-        <v>2.0286</v>
-      </c>
-      <c r="M61" t="n">
-        <v>1.8934</v>
-      </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>OPUS AC 9% BKR-NVDA-ROG  04.03.2027</t>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>VO AC 8.5% UBER-JPM-MA  01.02.2027</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ROG</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>JPMorgan Chase</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3897,49 +3525,43 @@
         <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>118325.081</v>
+        <v>349629.2302</v>
       </c>
       <c r="F62" t="n">
-        <v>0.6762</v>
+        <v>1.998</v>
       </c>
       <c r="G62" t="n">
-        <v>0.6311</v>
+        <v>1.8649</v>
       </c>
       <c r="H62" t="n">
-        <v>-0.0451</v>
+        <v>-0.1331</v>
       </c>
       <c r="I62" t="n">
         <v>-6.664</v>
       </c>
       <c r="J62" t="n">
-        <v>-0.3763</v>
+        <v>-1.0209</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L62" t="n">
-        <v>2.0286</v>
-      </c>
-      <c r="M62" t="n">
-        <v>1.8934</v>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>OPUS AC 9% BKR-NVDA-ROG  04.03.2027</t>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>VO AC 8.5% UBER-JPM-MA  01.02.2027</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>UBER</t>
+          <t>HNR1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Hannover Re</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3951,49 +3573,43 @@
         <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>116543.0767</v>
+        <v>347205.7044</v>
       </c>
       <c r="F63" t="n">
-        <v>0.666</v>
+        <v>1.9842</v>
       </c>
       <c r="G63" t="n">
-        <v>0.6216</v>
+        <v>1.852</v>
       </c>
       <c r="H63" t="n">
-        <v>-0.0444</v>
+        <v>-0.1322</v>
       </c>
       <c r="I63" t="n">
         <v>-6.664</v>
       </c>
       <c r="J63" t="n">
-        <v>-0.3859</v>
+        <v>-1.0339</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L63" t="n">
-        <v>1.998</v>
-      </c>
-      <c r="M63" t="n">
-        <v>1.8649</v>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>VO AC 8.5% UBER-JPM-MA  01.02.2027</t>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>TCM AC 8.5% AIR-HNR1-LIN  18.11.2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>Linde</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -4005,49 +3621,43 @@
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>116543.0767</v>
+        <v>347205.7044</v>
       </c>
       <c r="F64" t="n">
-        <v>0.666</v>
+        <v>1.9842</v>
       </c>
       <c r="G64" t="n">
-        <v>0.6216</v>
+        <v>1.852</v>
       </c>
       <c r="H64" t="n">
-        <v>-0.0444</v>
+        <v>-0.1322</v>
       </c>
       <c r="I64" t="n">
         <v>-6.664</v>
       </c>
       <c r="J64" t="n">
-        <v>-0.3859</v>
+        <v>-1.0339</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L64" t="n">
-        <v>1.998</v>
-      </c>
-      <c r="M64" t="n">
-        <v>1.8649</v>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>VO AC 8.5% UBER-JPM-MA  01.02.2027</t>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>TCM AC 8.5% AIR-HNR1-LIN  18.11.2026</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>HNR1</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Hannover Re</t>
+          <t>Arista Networks</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4059,49 +3669,43 @@
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>115735.2348</v>
+        <v>268877.7084</v>
       </c>
       <c r="F65" t="n">
-        <v>0.6614</v>
+        <v>1.5366</v>
       </c>
       <c r="G65" t="n">
-        <v>0.6173</v>
+        <v>1.4342</v>
       </c>
       <c r="H65" t="n">
-        <v>-0.0441</v>
+        <v>-0.1024</v>
       </c>
       <c r="I65" t="n">
         <v>-6.664</v>
       </c>
       <c r="J65" t="n">
-        <v>-0.3902</v>
+        <v>-1.4517</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L65" t="n">
-        <v>1.9842</v>
-      </c>
-      <c r="M65" t="n">
-        <v>1.852</v>
-      </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>TCM AC 8.5% AIR-HNR1-LIN  18.11.2026</t>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>UBS AC 11.1% ANET-APH  04.08.2027</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Linde</t>
+          <t>Amphenol</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4113,37 +3717,31 @@
         <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>115735.2348</v>
+        <v>268877.7084</v>
       </c>
       <c r="F66" t="n">
-        <v>0.6614</v>
+        <v>1.5366</v>
       </c>
       <c r="G66" t="n">
-        <v>0.6173</v>
+        <v>1.4342</v>
       </c>
       <c r="H66" t="n">
-        <v>-0.0441</v>
+        <v>-0.1024</v>
       </c>
       <c r="I66" t="n">
         <v>-6.664</v>
       </c>
       <c r="J66" t="n">
-        <v>-0.3902</v>
+        <v>-1.4517</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L66" t="n">
-        <v>1.9842</v>
-      </c>
-      <c r="M66" t="n">
-        <v>1.852</v>
-      </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>TCM AC 8.5% AIR-HNR1-LIN  18.11.2026</t>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>UBS AC 11.1% ANET-APH  04.08.2027</t>
         </is>
       </c>
     </row>
@@ -4167,35 +3765,29 @@
         <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>89608.0828</v>
+        <v>268824.2483</v>
       </c>
       <c r="F67" t="n">
-        <v>0.5121</v>
+        <v>1.5363</v>
       </c>
       <c r="G67" t="n">
-        <v>0.478</v>
+        <v>1.4339</v>
       </c>
       <c r="H67" t="n">
-        <v>-0.0341</v>
+        <v>-0.1024</v>
       </c>
       <c r="I67" t="n">
         <v>-6.664</v>
       </c>
       <c r="J67" t="n">
-        <v>-0.5295</v>
+        <v>-1.4519</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L67" t="n">
-        <v>1.5363</v>
-      </c>
-      <c r="M67" t="n">
-        <v>1.4339</v>
-      </c>
-      <c r="N67" t="inlineStr">
+      <c r="L67" t="inlineStr">
         <is>
           <t>BIL AC 9.3% ASML-OR-DG  11.06.2027</t>
         </is>
@@ -4221,35 +3813,29 @@
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>87398.39750000001</v>
+        <v>262195.1926</v>
       </c>
       <c r="F68" t="n">
-        <v>0.4995</v>
+        <v>1.4984</v>
       </c>
       <c r="G68" t="n">
-        <v>0.4662</v>
+        <v>1.3985</v>
       </c>
       <c r="H68" t="n">
-        <v>-0.0333</v>
+        <v>-0.0999</v>
       </c>
       <c r="I68" t="n">
         <v>-6.664</v>
       </c>
       <c r="J68" t="n">
-        <v>-0.5413</v>
+        <v>-1.4873</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L68" t="n">
-        <v>1.4984</v>
-      </c>
-      <c r="M68" t="n">
-        <v>1.3985</v>
-      </c>
-      <c r="N68" t="inlineStr">
+      <c r="L68" t="inlineStr">
         <is>
           <t>AC 8.5% GEBN-GIVN-SREN  01.03.2027</t>
         </is>
@@ -4275,35 +3861,29 @@
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>87398.39750000001</v>
+        <v>262195.1926</v>
       </c>
       <c r="F69" t="n">
-        <v>0.4995</v>
+        <v>1.4984</v>
       </c>
       <c r="G69" t="n">
-        <v>0.4662</v>
+        <v>1.3985</v>
       </c>
       <c r="H69" t="n">
-        <v>-0.0333</v>
+        <v>-0.0999</v>
       </c>
       <c r="I69" t="n">
         <v>-6.664</v>
       </c>
       <c r="J69" t="n">
-        <v>-0.5413</v>
+        <v>-1.4873</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L69" t="n">
-        <v>1.4984</v>
-      </c>
-      <c r="M69" t="n">
-        <v>1.3985</v>
-      </c>
-      <c r="N69" t="inlineStr">
+      <c r="L69" t="inlineStr">
         <is>
           <t>AC 8.5% GEBN-GIVN-SREN  01.03.2027</t>
         </is>
@@ -4329,35 +3909,29 @@
         <v>1</v>
       </c>
       <c r="E70" t="n">
-        <v>87398.39750000001</v>
+        <v>262195.1926</v>
       </c>
       <c r="F70" t="n">
-        <v>0.4995</v>
+        <v>1.4984</v>
       </c>
       <c r="G70" t="n">
-        <v>0.4662</v>
+        <v>1.3985</v>
       </c>
       <c r="H70" t="n">
-        <v>-0.0333</v>
+        <v>-0.0999</v>
       </c>
       <c r="I70" t="n">
         <v>-6.664</v>
       </c>
       <c r="J70" t="n">
-        <v>-0.5413</v>
+        <v>-1.4873</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L70" t="n">
-        <v>1.4984</v>
-      </c>
-      <c r="M70" t="n">
-        <v>1.3985</v>
-      </c>
-      <c r="N70" t="inlineStr">
+      <c r="L70" t="inlineStr">
         <is>
           <t>AC 8.5% GEBN-GIVN-SREN  01.03.2027</t>
         </is>
@@ -4383,35 +3957,29 @@
         <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>85643.1234</v>
+        <v>256929.3701</v>
       </c>
       <c r="F71" t="n">
-        <v>0.4894</v>
+        <v>1.4683</v>
       </c>
       <c r="G71" t="n">
-        <v>0.4568</v>
+        <v>1.3704</v>
       </c>
       <c r="H71" t="n">
-        <v>-0.0326</v>
+        <v>-0.0978</v>
       </c>
       <c r="I71" t="n">
         <v>-6.664</v>
       </c>
       <c r="J71" t="n">
-        <v>-0.5507</v>
+        <v>-1.5154</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L71" t="n">
-        <v>1.4683</v>
-      </c>
-      <c r="M71" t="n">
-        <v>1.3704</v>
-      </c>
-      <c r="N71" t="inlineStr">
+      <c r="L71" t="inlineStr">
         <is>
           <t>POST AC 8.5% ABBN-NOVN-UB  29.09.2027</t>
         </is>
@@ -4437,35 +4005,29 @@
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>72022.671</v>
+        <v>216068.013</v>
       </c>
       <c r="F72" t="n">
-        <v>0.4116</v>
+        <v>1.2348</v>
       </c>
       <c r="G72" t="n">
-        <v>0.3842</v>
+        <v>1.1525</v>
       </c>
       <c r="H72" t="n">
-        <v>-0.0274</v>
+        <v>-0.0823</v>
       </c>
       <c r="I72" t="n">
         <v>-6.664</v>
       </c>
       <c r="J72" t="n">
-        <v>-0.6233</v>
+        <v>-1.7333</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L72" t="n">
-        <v>1.2348</v>
-      </c>
-      <c r="M72" t="n">
-        <v>1.1525</v>
-      </c>
-      <c r="N72" t="inlineStr">
+      <c r="L72" t="inlineStr">
         <is>
           <t>VO AC 8% HD-MA-WMT  01.03.2027</t>
         </is>
@@ -4491,35 +4053,29 @@
         <v>1</v>
       </c>
       <c r="E73" t="n">
-        <v>69423.9148</v>
+        <v>208271.7445</v>
       </c>
       <c r="F73" t="n">
-        <v>0.3967</v>
+        <v>1.1902</v>
       </c>
       <c r="G73" t="n">
-        <v>0.3703</v>
+        <v>1.1109</v>
       </c>
       <c r="H73" t="n">
-        <v>-0.0264</v>
+        <v>-0.0793</v>
       </c>
       <c r="I73" t="n">
         <v>-6.664</v>
       </c>
       <c r="J73" t="n">
-        <v>-0.6372</v>
+        <v>-1.7749</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L73" t="n">
-        <v>1.1902</v>
-      </c>
-      <c r="M73" t="n">
-        <v>1.1109</v>
-      </c>
-      <c r="N73" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>VO AC 8.5% BABA-1211-MELI  01.03.2027</t>
         </is>
@@ -4545,35 +4101,29 @@
         <v>1</v>
       </c>
       <c r="E74" t="n">
-        <v>69423.9148</v>
+        <v>208271.7445</v>
       </c>
       <c r="F74" t="n">
-        <v>0.3967</v>
+        <v>1.1902</v>
       </c>
       <c r="G74" t="n">
-        <v>0.3703</v>
+        <v>1.1109</v>
       </c>
       <c r="H74" t="n">
-        <v>-0.0264</v>
+        <v>-0.0793</v>
       </c>
       <c r="I74" t="n">
         <v>-6.664</v>
       </c>
       <c r="J74" t="n">
-        <v>-0.6372</v>
+        <v>-1.7749</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L74" t="n">
-        <v>1.1902</v>
-      </c>
-      <c r="M74" t="n">
-        <v>1.1109</v>
-      </c>
-      <c r="N74" t="inlineStr">
+      <c r="L74" t="inlineStr">
         <is>
           <t>VO AC 8.5% BABA-1211-MELI  01.03.2027</t>
         </is>
@@ -4599,35 +4149,29 @@
         <v>1</v>
       </c>
       <c r="E75" t="n">
-        <v>69423.9148</v>
+        <v>208271.7445</v>
       </c>
       <c r="F75" t="n">
-        <v>0.3967</v>
+        <v>1.1902</v>
       </c>
       <c r="G75" t="n">
-        <v>0.3703</v>
+        <v>1.1109</v>
       </c>
       <c r="H75" t="n">
-        <v>-0.0264</v>
+        <v>-0.0793</v>
       </c>
       <c r="I75" t="n">
         <v>-6.664</v>
       </c>
       <c r="J75" t="n">
-        <v>-0.6372</v>
+        <v>-1.7749</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L75" t="n">
-        <v>1.1902</v>
-      </c>
-      <c r="M75" t="n">
-        <v>1.1109</v>
-      </c>
-      <c r="N75" t="inlineStr">
+      <c r="L75" t="inlineStr">
         <is>
           <t>VO AC 8.5% BABA-1211-MELI  01.03.2027</t>
         </is>
@@ -4653,35 +4197,29 @@
         <v>1</v>
       </c>
       <c r="E76" t="n">
-        <v>67248.3847</v>
+        <v>201745.154</v>
       </c>
       <c r="F76" t="n">
-        <v>0.3843</v>
+        <v>1.1529</v>
       </c>
       <c r="G76" t="n">
-        <v>0.3587</v>
+        <v>1.0761</v>
       </c>
       <c r="H76" t="n">
-        <v>-0.0256</v>
+        <v>-0.07679999999999999</v>
       </c>
       <c r="I76" t="n">
         <v>-6.664</v>
       </c>
       <c r="J76" t="n">
-        <v>-0.6488</v>
+        <v>-1.8097</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L76" t="n">
-        <v>1.1529</v>
-      </c>
-      <c r="M76" t="n">
-        <v>1.0761</v>
-      </c>
-      <c r="N76" t="inlineStr">
+      <c r="L76" t="inlineStr">
         <is>
           <t>TCM AC 9.35% RACE-CFR-RMS  25.02.2027</t>
         </is>
@@ -4707,35 +4245,29 @@
         <v>1</v>
       </c>
       <c r="E77" t="n">
-        <v>67248.3847</v>
+        <v>201745.154</v>
       </c>
       <c r="F77" t="n">
-        <v>0.3843</v>
+        <v>1.1529</v>
       </c>
       <c r="G77" t="n">
-        <v>0.3587</v>
+        <v>1.0761</v>
       </c>
       <c r="H77" t="n">
-        <v>-0.0256</v>
+        <v>-0.07679999999999999</v>
       </c>
       <c r="I77" t="n">
         <v>-6.664</v>
       </c>
       <c r="J77" t="n">
-        <v>-0.6488</v>
+        <v>-1.8097</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L77" t="n">
-        <v>1.1529</v>
-      </c>
-      <c r="M77" t="n">
-        <v>1.0761</v>
-      </c>
-      <c r="N77" t="inlineStr">
+      <c r="L77" t="inlineStr">
         <is>
           <t>TCM AC 9.35% RACE-CFR-RMS  25.02.2027</t>
         </is>
@@ -4761,35 +4293,29 @@
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>67248.3847</v>
+        <v>201745.154</v>
       </c>
       <c r="F78" t="n">
-        <v>0.3843</v>
+        <v>1.1529</v>
       </c>
       <c r="G78" t="n">
-        <v>0.3587</v>
+        <v>1.0761</v>
       </c>
       <c r="H78" t="n">
-        <v>-0.0256</v>
+        <v>-0.07679999999999999</v>
       </c>
       <c r="I78" t="n">
         <v>-6.664</v>
       </c>
       <c r="J78" t="n">
-        <v>-0.6488</v>
+        <v>-1.8097</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L78" t="n">
-        <v>1.1529</v>
-      </c>
-      <c r="M78" t="n">
-        <v>1.0761</v>
-      </c>
-      <c r="N78" t="inlineStr">
+      <c r="L78" t="inlineStr">
         <is>
           <t>TCM AC 9.35% RACE-CFR-RMS  25.02.2027</t>
         </is>
@@ -4815,35 +4341,29 @@
         <v>1</v>
       </c>
       <c r="E79" t="n">
-        <v>66676.6583</v>
+        <v>200029.975</v>
       </c>
       <c r="F79" t="n">
-        <v>0.381</v>
+        <v>1.1431</v>
       </c>
       <c r="G79" t="n">
-        <v>0.3556</v>
+        <v>1.0669</v>
       </c>
       <c r="H79" t="n">
-        <v>-0.0254</v>
+        <v>-0.0762</v>
       </c>
       <c r="I79" t="n">
         <v>-6.664</v>
       </c>
       <c r="J79" t="n">
-        <v>-0.6518</v>
+        <v>-1.8189</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L79" t="n">
-        <v>1.1431</v>
-      </c>
-      <c r="M79" t="n">
-        <v>1.0669</v>
-      </c>
-      <c r="N79" t="inlineStr">
+      <c r="L79" t="inlineStr">
         <is>
           <t>EFG AC 8.5% BKNG-CVX-MCD  01.03.2027</t>
         </is>
@@ -4869,35 +4389,29 @@
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>66676.6583</v>
+        <v>200029.975</v>
       </c>
       <c r="F80" t="n">
-        <v>0.381</v>
+        <v>1.1431</v>
       </c>
       <c r="G80" t="n">
-        <v>0.3556</v>
+        <v>1.0669</v>
       </c>
       <c r="H80" t="n">
-        <v>-0.0254</v>
+        <v>-0.0762</v>
       </c>
       <c r="I80" t="n">
         <v>-6.664</v>
       </c>
       <c r="J80" t="n">
-        <v>-0.6518</v>
+        <v>-1.8189</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
           <t>Underweight</t>
         </is>
       </c>
-      <c r="L80" t="n">
-        <v>1.1431</v>
-      </c>
-      <c r="M80" t="n">
-        <v>1.0669</v>
-      </c>
-      <c r="N80" t="inlineStr">
+      <c r="L80" t="inlineStr">
         <is>
           <t>EFG AC 8.5% BKNG-CVX-MCD  01.03.2027</t>
         </is>
@@ -4918,7 +4432,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -4932,7 +4446,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Look-through EUR</t>
+          <t>Exposure EUR</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -4958,16 +4472,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>399026.3875</v>
+        <v>1197079.1625</v>
       </c>
       <c r="C2" t="n">
-        <v>2.2803</v>
+        <v>6.841</v>
       </c>
       <c r="D2" t="n">
-        <v>2.1284</v>
+        <v>6.3851</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.152</v>
+        <v>-0.4559</v>
       </c>
     </row>
     <row r="3">
@@ -4977,16 +4491,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3429860.4848</v>
+        <v>10289581.4544</v>
       </c>
       <c r="C3" t="n">
-        <v>19.6008</v>
+        <v>58.8023</v>
       </c>
       <c r="D3" t="n">
-        <v>18.2946</v>
+        <v>54.8837</v>
       </c>
       <c r="E3" t="n">
-        <v>-1.3062</v>
+        <v>-3.9186</v>
       </c>
     </row>
     <row r="4">
@@ -4996,16 +4510,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11092806.2049</v>
+        <v>31255036.2042</v>
       </c>
       <c r="C4" t="n">
-        <v>63.3925</v>
+        <v>178.6143</v>
       </c>
       <c r="D4" t="n">
-        <v>59.168</v>
+        <v>166.7114</v>
       </c>
       <c r="E4" t="n">
-        <v>-4.2245</v>
+        <v>-11.9029</v>
       </c>
     </row>
   </sheetData>

</xml_diff>